<commit_message>
Aggiunti Log per visualizzazione migliore su console
</commit_message>
<xml_diff>
--- a/src/test/resources/SportelloCittadino/Sportello UT - Test Automatici.xlsx
+++ b/src/test/resources/SportelloCittadino/Sportello UT - Test Automatici.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="178">
   <si>
     <t>Classe_Test</t>
   </si>
@@ -541,6 +541,27 @@
   </si>
   <si>
     <t>15/05/2025 13:04:07</t>
+  </si>
+  <si>
+    <t>26/05/2025 11:44:57</t>
+  </si>
+  <si>
+    <t>26/05/2025 11:55:16</t>
+  </si>
+  <si>
+    <t>26/05/2025 11:57:15</t>
+  </si>
+  <si>
+    <t>26/05/2025 12:10:20</t>
+  </si>
+  <si>
+    <t>26/05/2025 12:15:13</t>
+  </si>
+  <si>
+    <t>26/05/2025 12:33:16</t>
+  </si>
+  <si>
+    <t>26/05/2025 12:45:16</t>
   </si>
 </sst>
 </file>
@@ -1239,7 +1260,7 @@
         <v>45</v>
       </c>
       <c r="H2" t="s" s="5">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>13</v>
@@ -1289,7 +1310,7 @@
         <v>45</v>
       </c>
       <c r="H3" t="s" s="5">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>13</v>
@@ -1339,7 +1360,7 @@
         <v>51</v>
       </c>
       <c r="H4" t="s" s="5">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Leggere modifiche al codice
</commit_message>
<xml_diff>
--- a/src/test/resources/SportelloCittadino/Sportello UT - Test Automatici.xlsx
+++ b/src/test/resources/SportelloCittadino/Sportello UT - Test Automatici.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="185">
   <si>
     <t>Classe_Test</t>
   </si>
@@ -562,6 +562,27 @@
   </si>
   <si>
     <t>26/05/2025 12:45:16</t>
+  </si>
+  <si>
+    <t>04/06/2025 10:05:56</t>
+  </si>
+  <si>
+    <t>04/06/2025 10:09:23</t>
+  </si>
+  <si>
+    <t>04/06/2025 10:15:29</t>
+  </si>
+  <si>
+    <t>04/06/2025 10:18:05</t>
+  </si>
+  <si>
+    <t>04/06/2025 10:20:57</t>
+  </si>
+  <si>
+    <t>04/06/2025 10:23:37</t>
+  </si>
+  <si>
+    <t>04/06/2025 10:31:15</t>
   </si>
 </sst>
 </file>
@@ -1260,7 +1281,7 @@
         <v>45</v>
       </c>
       <c r="H2" t="s" s="5">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>13</v>
@@ -1354,13 +1375,13 @@
         <v>11</v>
       </c>
       <c r="F4" t="s" s="5">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="G4" t="s" s="5">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H4" t="s" s="5">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Vediamo se funziona tutto
</commit_message>
<xml_diff>
--- a/src/test/resources/SportelloCittadino/Sportello UT - Test Automatici.xlsx
+++ b/src/test/resources/SportelloCittadino/Sportello UT - Test Automatici.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="201">
   <si>
     <t>Classe_Test</t>
   </si>
@@ -583,6 +583,54 @@
   </si>
   <si>
     <t>04/06/2025 10:31:15</t>
+  </si>
+  <si>
+    <t>09/06/2025 12:45:23</t>
+  </si>
+  <si>
+    <t>09/06/2025 12:49:17</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:13:43</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:15:55</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:26:46</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:30:02</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:32:31</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:39:16</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:41:19</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:43:44</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:45:37</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:47:45</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:48:32</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:52:31</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:53:41</t>
+  </si>
+  <si>
+    <t>09/06/2025 14:54:45</t>
   </si>
 </sst>
 </file>
@@ -1381,7 +1429,7 @@
         <v>45</v>
       </c>
       <c r="H4" t="s" s="5">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>13</v>
@@ -1431,7 +1479,7 @@
         <v>45</v>
       </c>
       <c r="H5" t="s" s="5">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>13</v>
@@ -1481,7 +1529,7 @@
         <v>45</v>
       </c>
       <c r="H6" t="s" s="5">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>13</v>
@@ -1525,13 +1573,13 @@
         <v>11</v>
       </c>
       <c r="F7" t="s" s="5">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="G7" t="s" s="5">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H7" t="s" s="5">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>13</v>
@@ -1575,13 +1623,13 @@
         <v>11</v>
       </c>
       <c r="F8" t="s" s="5">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="G8" t="s" s="5">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H8" t="s" s="5">
-        <v>170</v>
+        <v>194</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>13</v>
@@ -1625,13 +1673,13 @@
         <v>11</v>
       </c>
       <c r="F9" t="s" s="5">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="G9" t="s" s="5">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H9" t="s" s="5">
-        <v>153</v>
+        <v>195</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>13</v>
@@ -1675,13 +1723,13 @@
         <v>11</v>
       </c>
       <c r="F10" t="s" s="5">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="G10" t="s" s="5">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H10" t="s" s="5">
-        <v>154</v>
+        <v>196</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>13</v>
@@ -1725,13 +1773,13 @@
         <v>11</v>
       </c>
       <c r="F11" t="s" s="5">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="G11" t="s" s="5">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="H11" t="s" s="5">
-        <v>155</v>
+        <v>200</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>13</v>

</xml_diff>